<commit_message>
add roster batch import
</commit_message>
<xml_diff>
--- a/backend/assessment_bank_exports/思政试卷_第1份.xlsx
+++ b/backend/assessment_bank_exports/思政试卷_第1份.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CoWorkProjects\IntelligentMoralEducationWhole-processSystem1.0\backend\assessment_bank_exports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luoxu\.codex\worktrees\2c1f\IntelligentMoralEducationWhole-processSystem1.0\backend\assessment_bank_exports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A7A39F1-803D-4DBC-8915-D9ABC76B6325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304C1D25-001C-423A-A341-2291C57B78DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5295" yWindow="1935" windowWidth="28800" windowHeight="15420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4380" yWindow="3150" windowWidth="25365" windowHeight="15420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="262">
   <si>
     <t>说明</t>
   </si>
@@ -802,6 +802,14 @@
   </si>
   <si>
     <t>虚拟仿真训练提升医德实践能力。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>A</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>A,B,C,D</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1435,7 +1443,9 @@
       <c r="AE2" s="2"/>
       <c r="AF2" s="2"/>
       <c r="AG2" s="2"/>
-      <c r="AH2" s="2"/>
+      <c r="AH2" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI2" s="2">
         <v>2</v>
       </c>
@@ -1499,7 +1509,9 @@
       <c r="AE3" s="2"/>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
-      <c r="AH3" s="2"/>
+      <c r="AH3" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI3" s="2">
         <v>2</v>
       </c>
@@ -1563,7 +1575,9 @@
       <c r="AE4" s="2"/>
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
-      <c r="AH4" s="2"/>
+      <c r="AH4" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI4" s="2">
         <v>2</v>
       </c>
@@ -1627,7 +1641,9 @@
       <c r="AE5" s="2"/>
       <c r="AF5" s="2"/>
       <c r="AG5" s="2"/>
-      <c r="AH5" s="2"/>
+      <c r="AH5" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI5" s="2">
         <v>2</v>
       </c>
@@ -1691,7 +1707,9 @@
       <c r="AE6" s="2"/>
       <c r="AF6" s="2"/>
       <c r="AG6" s="2"/>
-      <c r="AH6" s="2"/>
+      <c r="AH6" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI6" s="2">
         <v>2</v>
       </c>
@@ -1755,7 +1773,9 @@
       <c r="AE7" s="2"/>
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
-      <c r="AH7" s="2"/>
+      <c r="AH7" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI7" s="2">
         <v>2</v>
       </c>
@@ -1819,7 +1839,9 @@
       <c r="AE8" s="2"/>
       <c r="AF8" s="2"/>
       <c r="AG8" s="2"/>
-      <c r="AH8" s="2"/>
+      <c r="AH8" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI8" s="2">
         <v>2</v>
       </c>
@@ -1883,7 +1905,9 @@
       <c r="AE9" s="2"/>
       <c r="AF9" s="2"/>
       <c r="AG9" s="2"/>
-      <c r="AH9" s="2"/>
+      <c r="AH9" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI9" s="2">
         <v>2</v>
       </c>
@@ -1947,7 +1971,9 @@
       <c r="AE10" s="2"/>
       <c r="AF10" s="2"/>
       <c r="AG10" s="2"/>
-      <c r="AH10" s="2"/>
+      <c r="AH10" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI10" s="2">
         <v>2</v>
       </c>
@@ -2011,7 +2037,9 @@
       <c r="AE11" s="2"/>
       <c r="AF11" s="2"/>
       <c r="AG11" s="2"/>
-      <c r="AH11" s="2"/>
+      <c r="AH11" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI11" s="2">
         <v>2</v>
       </c>
@@ -2075,7 +2103,9 @@
       <c r="AE12" s="2"/>
       <c r="AF12" s="2"/>
       <c r="AG12" s="2"/>
-      <c r="AH12" s="2"/>
+      <c r="AH12" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI12" s="2">
         <v>2</v>
       </c>
@@ -2139,7 +2169,9 @@
       <c r="AE13" s="2"/>
       <c r="AF13" s="2"/>
       <c r="AG13" s="2"/>
-      <c r="AH13" s="2"/>
+      <c r="AH13" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI13" s="2">
         <v>2</v>
       </c>
@@ -2203,7 +2235,9 @@
       <c r="AE14" s="2"/>
       <c r="AF14" s="2"/>
       <c r="AG14" s="2"/>
-      <c r="AH14" s="2"/>
+      <c r="AH14" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI14" s="2">
         <v>2</v>
       </c>
@@ -2267,7 +2301,9 @@
       <c r="AE15" s="2"/>
       <c r="AF15" s="2"/>
       <c r="AG15" s="2"/>
-      <c r="AH15" s="2"/>
+      <c r="AH15" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI15" s="2">
         <v>2</v>
       </c>
@@ -2327,7 +2363,9 @@
       <c r="AE16" s="2"/>
       <c r="AF16" s="2"/>
       <c r="AG16" s="2"/>
-      <c r="AH16" s="2"/>
+      <c r="AH16" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI16" s="2">
         <v>2</v>
       </c>
@@ -2391,7 +2429,9 @@
       <c r="AE17" s="2"/>
       <c r="AF17" s="2"/>
       <c r="AG17" s="2"/>
-      <c r="AH17" s="2"/>
+      <c r="AH17" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI17" s="2">
         <v>2</v>
       </c>
@@ -2455,7 +2495,9 @@
       <c r="AE18" s="2"/>
       <c r="AF18" s="2"/>
       <c r="AG18" s="2"/>
-      <c r="AH18" s="2"/>
+      <c r="AH18" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI18" s="2">
         <v>2</v>
       </c>
@@ -2519,7 +2561,9 @@
       <c r="AE19" s="2"/>
       <c r="AF19" s="2"/>
       <c r="AG19" s="2"/>
-      <c r="AH19" s="2"/>
+      <c r="AH19" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI19" s="2">
         <v>2</v>
       </c>
@@ -2583,7 +2627,9 @@
       <c r="AE20" s="2"/>
       <c r="AF20" s="2"/>
       <c r="AG20" s="2"/>
-      <c r="AH20" s="2"/>
+      <c r="AH20" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI20" s="2">
         <v>2</v>
       </c>
@@ -2647,7 +2693,9 @@
       <c r="AE21" s="2"/>
       <c r="AF21" s="2"/>
       <c r="AG21" s="2"/>
-      <c r="AH21" s="2"/>
+      <c r="AH21" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI21" s="2">
         <v>2</v>
       </c>
@@ -2711,7 +2759,9 @@
       <c r="AE22" s="2"/>
       <c r="AF22" s="2"/>
       <c r="AG22" s="2"/>
-      <c r="AH22" s="2"/>
+      <c r="AH22" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI22" s="2">
         <v>2</v>
       </c>
@@ -2775,7 +2825,9 @@
       <c r="AE23" s="2"/>
       <c r="AF23" s="2"/>
       <c r="AG23" s="2"/>
-      <c r="AH23" s="2"/>
+      <c r="AH23" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI23" s="2">
         <v>2</v>
       </c>
@@ -2839,7 +2891,9 @@
       <c r="AE24" s="2"/>
       <c r="AF24" s="2"/>
       <c r="AG24" s="2"/>
-      <c r="AH24" s="2"/>
+      <c r="AH24" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI24" s="2">
         <v>2</v>
       </c>
@@ -2903,7 +2957,9 @@
       <c r="AE25" s="2"/>
       <c r="AF25" s="2"/>
       <c r="AG25" s="2"/>
-      <c r="AH25" s="2"/>
+      <c r="AH25" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI25" s="2">
         <v>2</v>
       </c>
@@ -2967,7 +3023,9 @@
       <c r="AE26" s="2"/>
       <c r="AF26" s="2"/>
       <c r="AG26" s="2"/>
-      <c r="AH26" s="2"/>
+      <c r="AH26" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="AI26" s="2">
         <v>2</v>
       </c>
@@ -3031,7 +3089,9 @@
       <c r="AE27" s="2"/>
       <c r="AF27" s="2"/>
       <c r="AG27" s="2"/>
-      <c r="AH27" s="2"/>
+      <c r="AH27" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI27" s="2">
         <v>2</v>
       </c>
@@ -3095,7 +3155,9 @@
       <c r="AE28" s="2"/>
       <c r="AF28" s="2"/>
       <c r="AG28" s="2"/>
-      <c r="AH28" s="2"/>
+      <c r="AH28" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI28" s="2">
         <v>2</v>
       </c>
@@ -3159,7 +3221,9 @@
       <c r="AE29" s="2"/>
       <c r="AF29" s="2"/>
       <c r="AG29" s="2"/>
-      <c r="AH29" s="2"/>
+      <c r="AH29" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI29" s="2">
         <v>2</v>
       </c>
@@ -3223,7 +3287,9 @@
       <c r="AE30" s="2"/>
       <c r="AF30" s="2"/>
       <c r="AG30" s="2"/>
-      <c r="AH30" s="2"/>
+      <c r="AH30" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI30" s="2">
         <v>2</v>
       </c>
@@ -3287,7 +3353,9 @@
       <c r="AE31" s="2"/>
       <c r="AF31" s="2"/>
       <c r="AG31" s="2"/>
-      <c r="AH31" s="2"/>
+      <c r="AH31" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI31" s="2">
         <v>2</v>
       </c>
@@ -3351,7 +3419,9 @@
       <c r="AE32" s="2"/>
       <c r="AF32" s="2"/>
       <c r="AG32" s="2"/>
-      <c r="AH32" s="2"/>
+      <c r="AH32" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI32" s="2">
         <v>2</v>
       </c>
@@ -3415,7 +3485,9 @@
       <c r="AE33" s="2"/>
       <c r="AF33" s="2"/>
       <c r="AG33" s="2"/>
-      <c r="AH33" s="2"/>
+      <c r="AH33" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI33" s="2">
         <v>2</v>
       </c>
@@ -3479,7 +3551,9 @@
       <c r="AE34" s="2"/>
       <c r="AF34" s="2"/>
       <c r="AG34" s="2"/>
-      <c r="AH34" s="2"/>
+      <c r="AH34" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI34" s="2">
         <v>2</v>
       </c>
@@ -3543,7 +3617,9 @@
       <c r="AE35" s="2"/>
       <c r="AF35" s="2"/>
       <c r="AG35" s="2"/>
-      <c r="AH35" s="2"/>
+      <c r="AH35" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI35" s="2">
         <v>2</v>
       </c>
@@ -3607,7 +3683,9 @@
       <c r="AE36" s="2"/>
       <c r="AF36" s="2"/>
       <c r="AG36" s="2"/>
-      <c r="AH36" s="2"/>
+      <c r="AH36" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI36" s="2">
         <v>2</v>
       </c>
@@ -3671,7 +3749,9 @@
       <c r="AE37" s="2"/>
       <c r="AF37" s="2"/>
       <c r="AG37" s="2"/>
-      <c r="AH37" s="2"/>
+      <c r="AH37" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI37" s="2">
         <v>2</v>
       </c>
@@ -3735,7 +3815,9 @@
       <c r="AE38" s="2"/>
       <c r="AF38" s="2"/>
       <c r="AG38" s="2"/>
-      <c r="AH38" s="2"/>
+      <c r="AH38" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI38" s="2">
         <v>2</v>
       </c>
@@ -3799,7 +3881,9 @@
       <c r="AE39" s="2"/>
       <c r="AF39" s="2"/>
       <c r="AG39" s="2"/>
-      <c r="AH39" s="2"/>
+      <c r="AH39" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI39" s="2">
         <v>2</v>
       </c>
@@ -3863,7 +3947,9 @@
       <c r="AE40" s="2"/>
       <c r="AF40" s="2"/>
       <c r="AG40" s="2"/>
-      <c r="AH40" s="2"/>
+      <c r="AH40" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI40" s="2">
         <v>2</v>
       </c>
@@ -3927,7 +4013,9 @@
       <c r="AE41" s="2"/>
       <c r="AF41" s="2"/>
       <c r="AG41" s="2"/>
-      <c r="AH41" s="2"/>
+      <c r="AH41" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="AI41" s="2">
         <v>2</v>
       </c>
@@ -3987,7 +4075,9 @@
       <c r="AE42" s="2"/>
       <c r="AF42" s="2"/>
       <c r="AG42" s="2"/>
-      <c r="AH42" s="2"/>
+      <c r="AH42" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI42" s="2">
         <v>2</v>
       </c>
@@ -4047,7 +4137,9 @@
       <c r="AE43" s="2"/>
       <c r="AF43" s="2"/>
       <c r="AG43" s="2"/>
-      <c r="AH43" s="2"/>
+      <c r="AH43" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AI43" s="2">
         <v>2</v>
       </c>
@@ -4107,7 +4199,9 @@
       <c r="AE44" s="2"/>
       <c r="AF44" s="2"/>
       <c r="AG44" s="2"/>
-      <c r="AH44" s="2"/>
+      <c r="AH44" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI44" s="2">
         <v>2</v>
       </c>
@@ -4167,7 +4261,9 @@
       <c r="AE45" s="2"/>
       <c r="AF45" s="2"/>
       <c r="AG45" s="2"/>
-      <c r="AH45" s="2"/>
+      <c r="AH45" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI45" s="2">
         <v>2</v>
       </c>
@@ -4227,7 +4323,9 @@
       <c r="AE46" s="2"/>
       <c r="AF46" s="2"/>
       <c r="AG46" s="2"/>
-      <c r="AH46" s="2"/>
+      <c r="AH46" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI46" s="2">
         <v>2</v>
       </c>
@@ -4287,7 +4385,9 @@
       <c r="AE47" s="2"/>
       <c r="AF47" s="2"/>
       <c r="AG47" s="2"/>
-      <c r="AH47" s="2"/>
+      <c r="AH47" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI47" s="2">
         <v>2</v>
       </c>
@@ -4347,7 +4447,9 @@
       <c r="AE48" s="2"/>
       <c r="AF48" s="2"/>
       <c r="AG48" s="2"/>
-      <c r="AH48" s="2"/>
+      <c r="AH48" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI48" s="2">
         <v>2</v>
       </c>
@@ -4407,7 +4509,9 @@
       <c r="AE49" s="2"/>
       <c r="AF49" s="2"/>
       <c r="AG49" s="2"/>
-      <c r="AH49" s="2"/>
+      <c r="AH49" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI49" s="2">
         <v>2</v>
       </c>
@@ -4467,7 +4571,9 @@
       <c r="AE50" s="2"/>
       <c r="AF50" s="2"/>
       <c r="AG50" s="2"/>
-      <c r="AH50" s="2"/>
+      <c r="AH50" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI50" s="2">
         <v>2</v>
       </c>
@@ -4527,7 +4633,9 @@
       <c r="AE51" s="2"/>
       <c r="AF51" s="2"/>
       <c r="AG51" s="2"/>
-      <c r="AH51" s="2"/>
+      <c r="AH51" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="AI51" s="2">
         <v>2</v>
       </c>

</xml_diff>